<commit_message>
now with Kanemura, plus manuscript draft
</commit_message>
<xml_diff>
--- a/Kappa_scoring/Gold_Standard_Overview.xlsx
+++ b/Kappa_scoring/Gold_Standard_Overview.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sem.l.kampman/Documents/GitHub/quips/quips_private/Kappa_scoring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{057A86BC-18D4-1049-98C1-CD3CF1ED1414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33C54FED-0C66-C546-AACB-94352F9BF639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="840" windowWidth="38400" windowHeight="21600" xr2:uid="{4E3F4CC3-0563-A146-9958-FFCF367891F9}"/>
+    <workbookView xWindow="-38400" yWindow="1340" windowWidth="38400" windowHeight="21100" xr2:uid="{4E3F4CC3-0563-A146-9958-FFCF367891F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$95</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="114">
   <si>
     <t>Study_ID</t>
   </si>
@@ -378,6 +378,9 @@
   </si>
   <si>
     <t>D6_Risk</t>
+  </si>
+  <si>
+    <t>scoring_Kanemura_2015.json</t>
   </si>
 </sst>
 </file>
@@ -735,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADDBFD47-8216-464F-886C-C4D8DF61C6C4}">
-  <dimension ref="A1:J94"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="27.6640625" customWidth="1"/>
@@ -1068,7 +1071,7 @@
         <v>0</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>113</v>
       </c>
       <c r="C11" t="s">
         <v>26</v>
@@ -1080,7 +1083,7 @@
         <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G11" t="s">
         <v>6</v>
@@ -1089,10 +1092,10 @@
         <v>3</v>
       </c>
       <c r="I11" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J11" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -1100,7 +1103,7 @@
         <v>0</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
         <v>26</v>
@@ -1109,13 +1112,13 @@
         <v>2</v>
       </c>
       <c r="E12" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" t="s">
         <v>3</v>
       </c>
       <c r="G12" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H12" t="s">
         <v>3</v>
@@ -1124,7 +1127,7 @@
         <v>3</v>
       </c>
       <c r="J12" t="s">
-        <v>97</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -1132,7 +1135,7 @@
         <v>0</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
         <v>26</v>
@@ -1141,22 +1144,22 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G13" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H13" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I13" t="s">
         <v>3</v>
       </c>
       <c r="J13" t="s">
-        <v>6</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1164,7 +1167,7 @@
         <v>0</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
@@ -1173,19 +1176,19 @@
         <v>2</v>
       </c>
       <c r="E14" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G14" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H14" t="s">
         <v>6</v>
       </c>
       <c r="I14" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J14" t="s">
         <v>6</v>
@@ -1196,7 +1199,7 @@
         <v>0</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" t="s">
         <v>26</v>
@@ -1205,22 +1208,22 @@
         <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G15" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H15" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I15" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J15" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -1228,13 +1231,13 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16" t="s">
         <v>26</v>
       </c>
       <c r="D16" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" t="s">
         <v>3</v>
@@ -1243,16 +1246,16 @@
         <v>6</v>
       </c>
       <c r="G16" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H16" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I16" t="s">
         <v>3</v>
       </c>
       <c r="J16" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -1260,7 +1263,7 @@
         <v>0</v>
       </c>
       <c r="B17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17" t="s">
         <v>26</v>
@@ -1292,25 +1295,25 @@
         <v>0</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C18" t="s">
         <v>26</v>
       </c>
       <c r="D18" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G18" t="s">
         <v>6</v>
       </c>
       <c r="H18" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I18" t="s">
         <v>3</v>
@@ -1324,7 +1327,7 @@
         <v>0</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" t="s">
         <v>26</v>
@@ -1333,16 +1336,16 @@
         <v>2</v>
       </c>
       <c r="E19" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G19" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H19" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I19" t="s">
         <v>3</v>
@@ -1356,28 +1359,28 @@
         <v>0</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C20" t="s">
         <v>26</v>
       </c>
       <c r="D20" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" t="s">
         <v>3</v>
       </c>
       <c r="F20" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G20" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H20" t="s">
         <v>6</v>
       </c>
       <c r="I20" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J20" t="s">
         <v>6</v>
@@ -1388,7 +1391,7 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C21" t="s">
         <v>26</v>
@@ -1420,16 +1423,16 @@
         <v>0</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C22" t="s">
         <v>26</v>
       </c>
       <c r="D22" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F22" t="s">
         <v>3</v>
@@ -1441,7 +1444,7 @@
         <v>6</v>
       </c>
       <c r="I22" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J22" t="s">
         <v>6</v>
@@ -1452,16 +1455,16 @@
         <v>0</v>
       </c>
       <c r="B23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C23" t="s">
         <v>26</v>
       </c>
       <c r="D23" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E23" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F23" t="s">
         <v>3</v>
@@ -1473,7 +1476,7 @@
         <v>6</v>
       </c>
       <c r="I23" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J23" t="s">
         <v>6</v>
@@ -1484,10 +1487,10 @@
         <v>0</v>
       </c>
       <c r="B24" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C24" t="s">
-        <v>104</v>
+        <v>26</v>
       </c>
       <c r="D24" t="s">
         <v>6</v>
@@ -1496,7 +1499,7 @@
         <v>6</v>
       </c>
       <c r="F24" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G24" t="s">
         <v>6</v>
@@ -1516,7 +1519,7 @@
         <v>0</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C25" t="s">
         <v>104</v>
@@ -1548,7 +1551,7 @@
         <v>0</v>
       </c>
       <c r="B26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C26" t="s">
         <v>104</v>
@@ -1580,13 +1583,13 @@
         <v>0</v>
       </c>
       <c r="B27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C27" t="s">
         <v>104</v>
       </c>
       <c r="D27" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E27" t="s">
         <v>6</v>
@@ -1595,13 +1598,13 @@
         <v>6</v>
       </c>
       <c r="G27" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H27" t="s">
         <v>6</v>
       </c>
       <c r="I27" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J27" t="s">
         <v>6</v>
@@ -1612,7 +1615,7 @@
         <v>0</v>
       </c>
       <c r="B28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C28" t="s">
         <v>104</v>
@@ -1624,10 +1627,10 @@
         <v>6</v>
       </c>
       <c r="F28" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G28" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H28" t="s">
         <v>6</v>
@@ -1644,22 +1647,22 @@
         <v>0</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C29" t="s">
         <v>104</v>
       </c>
       <c r="D29" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" t="s">
         <v>6</v>
       </c>
       <c r="F29" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G29" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H29" t="s">
         <v>6</v>
@@ -1676,19 +1679,19 @@
         <v>0</v>
       </c>
       <c r="B30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C30" t="s">
         <v>104</v>
       </c>
       <c r="D30" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E30" t="s">
         <v>6</v>
       </c>
       <c r="F30" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G30" t="s">
         <v>3</v>
@@ -1697,7 +1700,7 @@
         <v>6</v>
       </c>
       <c r="I30" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J30" t="s">
         <v>6</v>
@@ -1708,31 +1711,31 @@
         <v>0</v>
       </c>
       <c r="B31" t="s">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="C31" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D31" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E31" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F31" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G31" t="s">
         <v>3</v>
       </c>
       <c r="H31" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I31" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J31" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
@@ -1740,7 +1743,7 @@
         <v>0</v>
       </c>
       <c r="B32" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C32" t="s">
         <v>105</v>
@@ -1749,7 +1752,7 @@
         <v>2</v>
       </c>
       <c r="E32" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F32" t="s">
         <v>2</v>
@@ -1761,7 +1764,7 @@
         <v>3</v>
       </c>
       <c r="I32" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J32" t="s">
         <v>3</v>
@@ -1772,7 +1775,7 @@
         <v>0</v>
       </c>
       <c r="B33" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C33" t="s">
         <v>105</v>
@@ -1793,7 +1796,7 @@
         <v>3</v>
       </c>
       <c r="I33" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J33" t="s">
         <v>3</v>
@@ -1804,7 +1807,7 @@
         <v>0</v>
       </c>
       <c r="B34" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C34" t="s">
         <v>105</v>
@@ -1813,7 +1816,7 @@
         <v>2</v>
       </c>
       <c r="E34" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F34" t="s">
         <v>2</v>
@@ -1828,7 +1831,7 @@
         <v>3</v>
       </c>
       <c r="J34" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
@@ -1836,7 +1839,7 @@
         <v>0</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C35" t="s">
         <v>105</v>
@@ -1868,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="B36" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C36" t="s">
         <v>105</v>
@@ -1892,7 +1895,7 @@
         <v>3</v>
       </c>
       <c r="J36" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
@@ -1900,7 +1903,7 @@
         <v>0</v>
       </c>
       <c r="B37" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C37" t="s">
         <v>105</v>
@@ -1924,7 +1927,7 @@
         <v>3</v>
       </c>
       <c r="J37" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
@@ -1932,7 +1935,7 @@
         <v>0</v>
       </c>
       <c r="B38" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C38" t="s">
         <v>105</v>
@@ -1956,7 +1959,7 @@
         <v>3</v>
       </c>
       <c r="J38" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
@@ -1964,7 +1967,7 @@
         <v>0</v>
       </c>
       <c r="B39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C39" t="s">
         <v>105</v>
@@ -1976,7 +1979,7 @@
         <v>3</v>
       </c>
       <c r="F39" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G39" t="s">
         <v>3</v>
@@ -1996,7 +1999,7 @@
         <v>0</v>
       </c>
       <c r="B40" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="C40" t="s">
         <v>105</v>
@@ -2005,10 +2008,10 @@
         <v>2</v>
       </c>
       <c r="E40" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F40" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G40" t="s">
         <v>3</v>
@@ -2020,7 +2023,7 @@
         <v>3</v>
       </c>
       <c r="J40" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
@@ -2028,7 +2031,7 @@
         <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="C41" t="s">
         <v>105</v>
@@ -2037,7 +2040,7 @@
         <v>2</v>
       </c>
       <c r="E41" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F41" t="s">
         <v>2</v>
@@ -2046,13 +2049,13 @@
         <v>3</v>
       </c>
       <c r="H41" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I41" t="s">
         <v>3</v>
       </c>
       <c r="J41" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
@@ -2060,10 +2063,10 @@
         <v>0</v>
       </c>
       <c r="B42" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="C42" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D42" t="s">
         <v>2</v>
@@ -2072,7 +2075,7 @@
         <v>3</v>
       </c>
       <c r="F42" t="s">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="G42" t="s">
         <v>3</v>
@@ -2092,7 +2095,7 @@
         <v>0</v>
       </c>
       <c r="B43" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C43" t="s">
         <v>106</v>
@@ -2110,13 +2113,13 @@
         <v>3</v>
       </c>
       <c r="H43" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I43" t="s">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="J43" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
@@ -2124,7 +2127,7 @@
         <v>0</v>
       </c>
       <c r="B44" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="C44" t="s">
         <v>106</v>
@@ -2133,22 +2136,22 @@
         <v>2</v>
       </c>
       <c r="E44" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F44" t="s">
         <v>100</v>
       </c>
       <c r="G44" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H44" t="s">
         <v>3</v>
       </c>
       <c r="I44" t="s">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="J44" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
@@ -2156,7 +2159,7 @@
         <v>0</v>
       </c>
       <c r="B45" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C45" t="s">
         <v>106</v>
@@ -2165,22 +2168,22 @@
         <v>2</v>
       </c>
       <c r="E45" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F45" t="s">
         <v>100</v>
       </c>
       <c r="G45" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H45" t="s">
         <v>3</v>
       </c>
       <c r="I45" t="s">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="J45" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
@@ -2188,7 +2191,7 @@
         <v>0</v>
       </c>
       <c r="B46" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C46" t="s">
         <v>106</v>
@@ -2197,7 +2200,7 @@
         <v>2</v>
       </c>
       <c r="E46" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F46" t="s">
         <v>100</v>
@@ -2206,13 +2209,13 @@
         <v>3</v>
       </c>
       <c r="H46" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I46" t="s">
         <v>100</v>
       </c>
       <c r="J46" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
@@ -2220,7 +2223,7 @@
         <v>0</v>
       </c>
       <c r="B47" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C47" t="s">
         <v>106</v>
@@ -2238,10 +2241,10 @@
         <v>3</v>
       </c>
       <c r="H47" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I47" t="s">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="J47" t="s">
         <v>2</v>
@@ -2252,7 +2255,7 @@
         <v>0</v>
       </c>
       <c r="B48" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C48" t="s">
         <v>106</v>
@@ -2261,7 +2264,7 @@
         <v>2</v>
       </c>
       <c r="E48" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F48" t="s">
         <v>100</v>
@@ -2270,13 +2273,13 @@
         <v>3</v>
       </c>
       <c r="H48" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I48" t="s">
         <v>3</v>
       </c>
       <c r="J48" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
@@ -2284,7 +2287,7 @@
         <v>0</v>
       </c>
       <c r="B49" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C49" t="s">
         <v>106</v>
@@ -2293,7 +2296,7 @@
         <v>2</v>
       </c>
       <c r="E49" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F49" t="s">
         <v>100</v>
@@ -2302,13 +2305,13 @@
         <v>3</v>
       </c>
       <c r="H49" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I49" t="s">
         <v>3</v>
       </c>
       <c r="J49" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
@@ -2316,7 +2319,7 @@
         <v>0</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C50" t="s">
         <v>106</v>
@@ -2325,7 +2328,7 @@
         <v>2</v>
       </c>
       <c r="E50" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F50" t="s">
         <v>100</v>
@@ -2334,10 +2337,10 @@
         <v>3</v>
       </c>
       <c r="H50" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I50" t="s">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="J50" t="s">
         <v>2</v>
@@ -2348,7 +2351,7 @@
         <v>0</v>
       </c>
       <c r="B51" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="C51" t="s">
         <v>106</v>
@@ -2366,13 +2369,13 @@
         <v>3</v>
       </c>
       <c r="H51" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I51" t="s">
         <v>100</v>
       </c>
       <c r="J51" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
@@ -2380,7 +2383,7 @@
         <v>0</v>
       </c>
       <c r="B52" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C52" t="s">
         <v>106</v>
@@ -2389,7 +2392,7 @@
         <v>2</v>
       </c>
       <c r="E52" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F52" t="s">
         <v>100</v>
@@ -2398,13 +2401,13 @@
         <v>3</v>
       </c>
       <c r="H52" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I52" t="s">
         <v>100</v>
       </c>
       <c r="J52" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
@@ -2412,7 +2415,7 @@
         <v>0</v>
       </c>
       <c r="B53" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C53" t="s">
         <v>106</v>
@@ -2430,13 +2433,13 @@
         <v>3</v>
       </c>
       <c r="H53" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I53" t="s">
         <v>100</v>
       </c>
       <c r="J53" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
@@ -2444,7 +2447,7 @@
         <v>0</v>
       </c>
       <c r="B54" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="C54" t="s">
         <v>106</v>
@@ -2453,13 +2456,13 @@
         <v>2</v>
       </c>
       <c r="E54" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F54" t="s">
         <v>100</v>
       </c>
       <c r="G54" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H54" t="s">
         <v>3</v>
@@ -2468,7 +2471,7 @@
         <v>100</v>
       </c>
       <c r="J54" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
@@ -2476,31 +2479,31 @@
         <v>0</v>
       </c>
       <c r="B55" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C55" t="s">
         <v>106</v>
       </c>
       <c r="D55" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E55" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F55" t="s">
         <v>100</v>
       </c>
       <c r="G55" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H55" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I55" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J55" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
@@ -2508,13 +2511,13 @@
         <v>0</v>
       </c>
       <c r="B56" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="C56" t="s">
         <v>106</v>
       </c>
       <c r="D56" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E56" t="s">
         <v>6</v>
@@ -2523,16 +2526,16 @@
         <v>100</v>
       </c>
       <c r="G56" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H56" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I56" t="s">
         <v>101</v>
       </c>
       <c r="J56" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
@@ -2540,16 +2543,16 @@
         <v>0</v>
       </c>
       <c r="B57" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C57" t="s">
         <v>106</v>
       </c>
       <c r="D57" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E57" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F57" t="s">
         <v>100</v>
@@ -2561,10 +2564,10 @@
         <v>3</v>
       </c>
       <c r="I57" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J57" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
@@ -2572,7 +2575,7 @@
         <v>0</v>
       </c>
       <c r="B58" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="C58" t="s">
         <v>106</v>
@@ -2581,7 +2584,7 @@
         <v>2</v>
       </c>
       <c r="E58" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F58" t="s">
         <v>100</v>
@@ -2596,7 +2599,7 @@
         <v>100</v>
       </c>
       <c r="J58" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
@@ -2604,7 +2607,7 @@
         <v>0</v>
       </c>
       <c r="B59" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="C59" t="s">
         <v>106</v>
@@ -2613,10 +2616,10 @@
         <v>2</v>
       </c>
       <c r="E59" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F59" t="s">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="G59" t="s">
         <v>3</v>
@@ -2636,7 +2639,7 @@
         <v>0</v>
       </c>
       <c r="B60" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C60" t="s">
         <v>106</v>
@@ -2645,13 +2648,13 @@
         <v>2</v>
       </c>
       <c r="E60" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F60" t="s">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="G60" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H60" t="s">
         <v>3</v>
@@ -2660,7 +2663,7 @@
         <v>100</v>
       </c>
       <c r="J60" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
@@ -2668,31 +2671,31 @@
         <v>0</v>
       </c>
       <c r="B61" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="C61" t="s">
         <v>106</v>
       </c>
       <c r="D61" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E61" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F61" t="s">
         <v>100</v>
       </c>
       <c r="G61" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H61" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I61" t="s">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="J61" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
@@ -2700,13 +2703,13 @@
         <v>0</v>
       </c>
       <c r="B62" t="s">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="C62" t="s">
         <v>106</v>
       </c>
       <c r="D62" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E62" t="s">
         <v>6</v>
@@ -2718,13 +2721,13 @@
         <v>6</v>
       </c>
       <c r="H62" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I62" t="s">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="J62" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
@@ -2732,7 +2735,7 @@
         <v>0</v>
       </c>
       <c r="B63" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C63" t="s">
         <v>106</v>
@@ -2741,22 +2744,22 @@
         <v>2</v>
       </c>
       <c r="E63" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F63" t="s">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="G63" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H63" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I63" t="s">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="J63" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
@@ -2764,7 +2767,7 @@
         <v>0</v>
       </c>
       <c r="B64" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C64" t="s">
         <v>106</v>
@@ -2776,19 +2779,19 @@
         <v>3</v>
       </c>
       <c r="F64" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G64" t="s">
         <v>3</v>
       </c>
       <c r="H64" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I64" t="s">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="J64" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.2">
@@ -2796,7 +2799,7 @@
         <v>0</v>
       </c>
       <c r="B65" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C65" t="s">
         <v>106</v>
@@ -2805,10 +2808,10 @@
         <v>2</v>
       </c>
       <c r="E65" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F65" t="s">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="G65" t="s">
         <v>3</v>
@@ -2828,7 +2831,7 @@
         <v>0</v>
       </c>
       <c r="B66" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="C66" t="s">
         <v>106</v>
@@ -2837,10 +2840,10 @@
         <v>2</v>
       </c>
       <c r="E66" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F66" t="s">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="G66" t="s">
         <v>3</v>
@@ -2860,7 +2863,7 @@
         <v>0</v>
       </c>
       <c r="B67" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="C67" t="s">
         <v>106</v>
@@ -2884,7 +2887,7 @@
         <v>100</v>
       </c>
       <c r="J67" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
@@ -2892,7 +2895,7 @@
         <v>0</v>
       </c>
       <c r="B68" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="C68" t="s">
         <v>106</v>
@@ -2904,16 +2907,16 @@
         <v>3</v>
       </c>
       <c r="F68" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G68" t="s">
         <v>3</v>
       </c>
       <c r="H68" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I68" t="s">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="J68" t="s">
         <v>3</v>
@@ -2924,7 +2927,7 @@
         <v>0</v>
       </c>
       <c r="B69" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C69" t="s">
         <v>106</v>
@@ -2936,7 +2939,7 @@
         <v>3</v>
       </c>
       <c r="F69" t="s">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="G69" t="s">
         <v>3</v>
@@ -2945,7 +2948,7 @@
         <v>6</v>
       </c>
       <c r="I69" t="s">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="J69" t="s">
         <v>3</v>
@@ -2956,31 +2959,31 @@
         <v>0</v>
       </c>
       <c r="B70" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="C70" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D70" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E70" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F70" t="s">
         <v>100</v>
       </c>
       <c r="G70" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H70" t="s">
         <v>6</v>
       </c>
       <c r="I70" t="s">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="J70" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
@@ -2988,13 +2991,13 @@
         <v>0</v>
       </c>
       <c r="B71" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C71" t="s">
         <v>107</v>
       </c>
       <c r="D71" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E71" t="s">
         <v>6</v>
@@ -3009,10 +3012,10 @@
         <v>6</v>
       </c>
       <c r="I71" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J71" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.2">
@@ -3020,13 +3023,13 @@
         <v>0</v>
       </c>
       <c r="B72" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C72" t="s">
         <v>107</v>
       </c>
       <c r="D72" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E72" t="s">
         <v>6</v>
@@ -3044,7 +3047,7 @@
         <v>3</v>
       </c>
       <c r="J72" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
@@ -3052,13 +3055,13 @@
         <v>0</v>
       </c>
       <c r="B73" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C73" t="s">
         <v>107</v>
       </c>
       <c r="D73" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E73" t="s">
         <v>6</v>
@@ -3076,7 +3079,7 @@
         <v>3</v>
       </c>
       <c r="J73" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
@@ -3084,13 +3087,13 @@
         <v>0</v>
       </c>
       <c r="B74" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C74" t="s">
         <v>107</v>
       </c>
       <c r="D74" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E74" t="s">
         <v>6</v>
@@ -3099,16 +3102,16 @@
         <v>100</v>
       </c>
       <c r="G74" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H74" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I74" t="s">
         <v>3</v>
       </c>
       <c r="J74" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
@@ -3116,13 +3119,13 @@
         <v>0</v>
       </c>
       <c r="B75" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="C75" t="s">
         <v>107</v>
       </c>
       <c r="D75" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E75" t="s">
         <v>6</v>
@@ -3131,7 +3134,7 @@
         <v>100</v>
       </c>
       <c r="G75" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H75" t="s">
         <v>3</v>
@@ -3148,7 +3151,7 @@
         <v>0</v>
       </c>
       <c r="B76" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="C76" t="s">
         <v>107</v>
@@ -3166,13 +3169,13 @@
         <v>6</v>
       </c>
       <c r="H76" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I76" t="s">
         <v>3</v>
       </c>
       <c r="J76" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.2">
@@ -3180,13 +3183,13 @@
         <v>0</v>
       </c>
       <c r="B77" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C77" t="s">
         <v>107</v>
       </c>
       <c r="D77" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E77" t="s">
         <v>6</v>
@@ -3201,10 +3204,10 @@
         <v>6</v>
       </c>
       <c r="I77" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J77" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.2">
@@ -3212,7 +3215,7 @@
         <v>0</v>
       </c>
       <c r="B78" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C78" t="s">
         <v>107</v>
@@ -3230,7 +3233,7 @@
         <v>6</v>
       </c>
       <c r="H78" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I78" t="s">
         <v>6</v>
@@ -3244,13 +3247,13 @@
         <v>0</v>
       </c>
       <c r="B79" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="C79" t="s">
         <v>107</v>
       </c>
       <c r="D79" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E79" t="s">
         <v>6</v>
@@ -3262,13 +3265,13 @@
         <v>6</v>
       </c>
       <c r="H79" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I79" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J79" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.2">
@@ -3276,13 +3279,13 @@
         <v>0</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="C80" t="s">
         <v>107</v>
       </c>
       <c r="D80" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E80" t="s">
         <v>6</v>
@@ -3297,10 +3300,10 @@
         <v>6</v>
       </c>
       <c r="I80" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J80" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.2">
@@ -3308,7 +3311,7 @@
         <v>0</v>
       </c>
       <c r="B81" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C81" t="s">
         <v>107</v>
@@ -3329,7 +3332,7 @@
         <v>6</v>
       </c>
       <c r="I81" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J81" t="s">
         <v>6</v>
@@ -3340,13 +3343,13 @@
         <v>0</v>
       </c>
       <c r="B82" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C82" t="s">
         <v>107</v>
       </c>
       <c r="D82" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E82" t="s">
         <v>6</v>
@@ -3364,7 +3367,7 @@
         <v>3</v>
       </c>
       <c r="J82" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.2">
@@ -3372,13 +3375,13 @@
         <v>0</v>
       </c>
       <c r="B83" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C83" t="s">
         <v>107</v>
       </c>
       <c r="D83" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E83" t="s">
         <v>6</v>
@@ -3393,10 +3396,10 @@
         <v>6</v>
       </c>
       <c r="I83" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J83" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
@@ -3404,13 +3407,13 @@
         <v>0</v>
       </c>
       <c r="B84" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C84" t="s">
         <v>107</v>
       </c>
       <c r="D84" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E84" t="s">
         <v>6</v>
@@ -3422,10 +3425,10 @@
         <v>6</v>
       </c>
       <c r="H84" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I84" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J84" t="s">
         <v>6</v>
@@ -3436,13 +3439,13 @@
         <v>0</v>
       </c>
       <c r="B85" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C85" t="s">
         <v>107</v>
       </c>
       <c r="D85" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E85" t="s">
         <v>6</v>
@@ -3454,10 +3457,10 @@
         <v>6</v>
       </c>
       <c r="H85" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I85" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J85" t="s">
         <v>6</v>
@@ -3468,7 +3471,7 @@
         <v>0</v>
       </c>
       <c r="B86" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="C86" t="s">
         <v>107</v>
@@ -3489,7 +3492,7 @@
         <v>6</v>
       </c>
       <c r="I86" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J86" t="s">
         <v>6</v>
@@ -3500,22 +3503,22 @@
         <v>0</v>
       </c>
       <c r="B87" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="C87" t="s">
         <v>107</v>
       </c>
       <c r="D87" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E87" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F87" t="s">
         <v>100</v>
       </c>
       <c r="G87" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H87" t="s">
         <v>6</v>
@@ -3532,25 +3535,25 @@
         <v>0</v>
       </c>
       <c r="B88" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C88" t="s">
         <v>107</v>
       </c>
       <c r="D88" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E88" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F88" t="s">
         <v>100</v>
       </c>
       <c r="G88" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H88" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I88" t="s">
         <v>3</v>
@@ -3564,13 +3567,13 @@
         <v>0</v>
       </c>
       <c r="B89" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C89" t="s">
         <v>107</v>
       </c>
       <c r="D89" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E89" t="s">
         <v>6</v>
@@ -3582,7 +3585,7 @@
         <v>6</v>
       </c>
       <c r="H89" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I89" t="s">
         <v>3</v>
@@ -3596,7 +3599,7 @@
         <v>0</v>
       </c>
       <c r="B90" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="C90" t="s">
         <v>107</v>
@@ -3617,7 +3620,7 @@
         <v>6</v>
       </c>
       <c r="I90" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J90" t="s">
         <v>6</v>
@@ -3628,7 +3631,7 @@
         <v>0</v>
       </c>
       <c r="B91" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="C91" t="s">
         <v>107</v>
@@ -3660,13 +3663,13 @@
         <v>0</v>
       </c>
       <c r="B92" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C92" t="s">
         <v>107</v>
       </c>
       <c r="D92" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E92" t="s">
         <v>6</v>
@@ -3678,10 +3681,10 @@
         <v>6</v>
       </c>
       <c r="H92" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I92" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J92" t="s">
         <v>6</v>
@@ -3692,7 +3695,7 @@
         <v>0</v>
       </c>
       <c r="B93" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C93" t="s">
         <v>107</v>
@@ -3710,13 +3713,13 @@
         <v>6</v>
       </c>
       <c r="H93" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I93" t="s">
         <v>3</v>
       </c>
       <c r="J93" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.2">
@@ -3724,25 +3727,25 @@
         <v>0</v>
       </c>
       <c r="B94" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C94" t="s">
         <v>107</v>
       </c>
       <c r="D94" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E94" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F94" t="s">
         <v>100</v>
       </c>
       <c r="G94" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H94" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I94" t="s">
         <v>3</v>
@@ -3751,8 +3754,40 @@
         <v>3</v>
       </c>
     </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>0</v>
+      </c>
+      <c r="B95" t="s">
+        <v>47</v>
+      </c>
+      <c r="C95" t="s">
+        <v>107</v>
+      </c>
+      <c r="D95" t="s">
+        <v>2</v>
+      </c>
+      <c r="E95" t="s">
+        <v>3</v>
+      </c>
+      <c r="F95" t="s">
+        <v>100</v>
+      </c>
+      <c r="G95" t="s">
+        <v>3</v>
+      </c>
+      <c r="H95" t="s">
+        <v>3</v>
+      </c>
+      <c r="I95" t="s">
+        <v>3</v>
+      </c>
+      <c r="J95" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J94" xr:uid="{ADDBFD47-8216-464F-886C-C4D8DF61C6C4}"/>
+  <autoFilter ref="A1:J95" xr:uid="{ADDBFD47-8216-464F-886C-C4D8DF61C6C4}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated figures, fixed small errors
</commit_message>
<xml_diff>
--- a/Kappa_scoring/Gold_Standard_Overview.xlsx
+++ b/Kappa_scoring/Gold_Standard_Overview.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sem.l.kampman/Documents/GitHub/quips/quips_private/Kappa_scoring/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33C54FED-0C66-C546-AACB-94352F9BF639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB880C9-4036-BE4A-B7FA-029598798D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="1340" windowWidth="38400" windowHeight="21100" xr2:uid="{4E3F4CC3-0563-A146-9958-FFCF367891F9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="113">
   <si>
     <t>Study_ID</t>
   </si>
@@ -330,9 +330,6 @@
   </si>
   <si>
     <t>scoring_McIntosh_2012.json</t>
-  </si>
-  <si>
-    <t>M</t>
   </si>
   <si>
     <t>Overall_Risk</t>
@@ -748,34 +745,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
         <v>102</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>103</v>
-      </c>
       <c r="D1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" t="s">
         <v>98</v>
       </c>
-      <c r="E1" t="s">
-        <v>99</v>
-      </c>
       <c r="F1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G1" t="s">
         <v>108</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>109</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>110</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>111</v>
-      </c>
-      <c r="J1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -1071,7 +1068,7 @@
         <v>0</v>
       </c>
       <c r="B11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C11" t="s">
         <v>26</v>
@@ -1159,7 +1156,7 @@
         <v>3</v>
       </c>
       <c r="J13" t="s">
-        <v>97</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1522,7 +1519,7 @@
         <v>27</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D25" t="s">
         <v>6</v>
@@ -1554,7 +1551,7 @@
         <v>28</v>
       </c>
       <c r="C26" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D26" t="s">
         <v>6</v>
@@ -1586,7 +1583,7 @@
         <v>29</v>
       </c>
       <c r="C27" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D27" t="s">
         <v>6</v>
@@ -1618,7 +1615,7 @@
         <v>30</v>
       </c>
       <c r="C28" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D28" t="s">
         <v>3</v>
@@ -1650,7 +1647,7 @@
         <v>31</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D29" t="s">
         <v>3</v>
@@ -1682,7 +1679,7 @@
         <v>32</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D30" t="s">
         <v>2</v>
@@ -1714,7 +1711,7 @@
         <v>33</v>
       </c>
       <c r="C31" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D31" t="s">
         <v>6</v>
@@ -1746,7 +1743,7 @@
         <v>68</v>
       </c>
       <c r="C32" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D32" t="s">
         <v>2</v>
@@ -1778,7 +1775,7 @@
         <v>60</v>
       </c>
       <c r="C33" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D33" t="s">
         <v>2</v>
@@ -1810,7 +1807,7 @@
         <v>62</v>
       </c>
       <c r="C34" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D34" t="s">
         <v>2</v>
@@ -1842,7 +1839,7 @@
         <v>67</v>
       </c>
       <c r="C35" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D35" t="s">
         <v>2</v>
@@ -1874,7 +1871,7 @@
         <v>66</v>
       </c>
       <c r="C36" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D36" t="s">
         <v>2</v>
@@ -1906,7 +1903,7 @@
         <v>59</v>
       </c>
       <c r="C37" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D37" t="s">
         <v>2</v>
@@ -1938,7 +1935,7 @@
         <v>61</v>
       </c>
       <c r="C38" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D38" t="s">
         <v>2</v>
@@ -1970,7 +1967,7 @@
         <v>65</v>
       </c>
       <c r="C39" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D39" t="s">
         <v>2</v>
@@ -2002,7 +1999,7 @@
         <v>64</v>
       </c>
       <c r="C40" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D40" t="s">
         <v>2</v>
@@ -2034,7 +2031,7 @@
         <v>19</v>
       </c>
       <c r="C41" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D41" t="s">
         <v>2</v>
@@ -2066,7 +2063,7 @@
         <v>63</v>
       </c>
       <c r="C42" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D42" t="s">
         <v>2</v>
@@ -2098,7 +2095,7 @@
         <v>89</v>
       </c>
       <c r="C43" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D43" t="s">
         <v>2</v>
@@ -2107,7 +2104,7 @@
         <v>3</v>
       </c>
       <c r="F43" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G43" t="s">
         <v>3</v>
@@ -2130,7 +2127,7 @@
         <v>82</v>
       </c>
       <c r="C44" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D44" t="s">
         <v>2</v>
@@ -2139,7 +2136,7 @@
         <v>3</v>
       </c>
       <c r="F44" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G44" t="s">
         <v>3</v>
@@ -2148,7 +2145,7 @@
         <v>3</v>
       </c>
       <c r="I44" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J44" t="s">
         <v>3</v>
@@ -2162,7 +2159,7 @@
         <v>70</v>
       </c>
       <c r="C45" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D45" t="s">
         <v>2</v>
@@ -2171,7 +2168,7 @@
         <v>6</v>
       </c>
       <c r="F45" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G45" t="s">
         <v>6</v>
@@ -2194,7 +2191,7 @@
         <v>74</v>
       </c>
       <c r="C46" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D46" t="s">
         <v>2</v>
@@ -2203,7 +2200,7 @@
         <v>3</v>
       </c>
       <c r="F46" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G46" t="s">
         <v>3</v>
@@ -2212,7 +2209,7 @@
         <v>3</v>
       </c>
       <c r="I46" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J46" t="s">
         <v>3</v>
@@ -2226,7 +2223,7 @@
         <v>73</v>
       </c>
       <c r="C47" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D47" t="s">
         <v>2</v>
@@ -2235,7 +2232,7 @@
         <v>6</v>
       </c>
       <c r="F47" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G47" t="s">
         <v>3</v>
@@ -2244,7 +2241,7 @@
         <v>6</v>
       </c>
       <c r="I47" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J47" t="s">
         <v>2</v>
@@ -2258,7 +2255,7 @@
         <v>75</v>
       </c>
       <c r="C48" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D48" t="s">
         <v>2</v>
@@ -2267,7 +2264,7 @@
         <v>6</v>
       </c>
       <c r="F48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G48" t="s">
         <v>3</v>
@@ -2290,7 +2287,7 @@
         <v>85</v>
       </c>
       <c r="C49" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D49" t="s">
         <v>2</v>
@@ -2299,7 +2296,7 @@
         <v>3</v>
       </c>
       <c r="F49" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G49" t="s">
         <v>3</v>
@@ -2322,7 +2319,7 @@
         <v>83</v>
       </c>
       <c r="C50" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D50" t="s">
         <v>2</v>
@@ -2331,7 +2328,7 @@
         <v>2</v>
       </c>
       <c r="F50" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G50" t="s">
         <v>3</v>
@@ -2354,7 +2351,7 @@
         <v>91</v>
       </c>
       <c r="C51" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D51" t="s">
         <v>2</v>
@@ -2363,7 +2360,7 @@
         <v>3</v>
       </c>
       <c r="F51" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G51" t="s">
         <v>3</v>
@@ -2372,7 +2369,7 @@
         <v>6</v>
       </c>
       <c r="I51" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J51" t="s">
         <v>2</v>
@@ -2386,7 +2383,7 @@
         <v>81</v>
       </c>
       <c r="C52" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D52" t="s">
         <v>2</v>
@@ -2395,7 +2392,7 @@
         <v>3</v>
       </c>
       <c r="F52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G52" t="s">
         <v>3</v>
@@ -2404,7 +2401,7 @@
         <v>3</v>
       </c>
       <c r="I52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J52" t="s">
         <v>3</v>
@@ -2418,7 +2415,7 @@
         <v>84</v>
       </c>
       <c r="C53" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D53" t="s">
         <v>2</v>
@@ -2427,7 +2424,7 @@
         <v>6</v>
       </c>
       <c r="F53" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G53" t="s">
         <v>3</v>
@@ -2436,7 +2433,7 @@
         <v>2</v>
       </c>
       <c r="I53" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J53" t="s">
         <v>2</v>
@@ -2450,7 +2447,7 @@
         <v>78</v>
       </c>
       <c r="C54" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D54" t="s">
         <v>2</v>
@@ -2459,7 +2456,7 @@
         <v>6</v>
       </c>
       <c r="F54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G54" t="s">
         <v>3</v>
@@ -2468,7 +2465,7 @@
         <v>3</v>
       </c>
       <c r="I54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J54" t="s">
         <v>3</v>
@@ -2482,7 +2479,7 @@
         <v>88</v>
       </c>
       <c r="C55" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D55" t="s">
         <v>2</v>
@@ -2491,7 +2488,7 @@
         <v>3</v>
       </c>
       <c r="F55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G55" t="s">
         <v>2</v>
@@ -2500,7 +2497,7 @@
         <v>3</v>
       </c>
       <c r="I55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J55" t="s">
         <v>2</v>
@@ -2514,7 +2511,7 @@
         <v>96</v>
       </c>
       <c r="C56" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D56" t="s">
         <v>6</v>
@@ -2523,16 +2520,16 @@
         <v>6</v>
       </c>
       <c r="F56" t="s">
+        <v>99</v>
+      </c>
+      <c r="G56" t="s">
+        <v>6</v>
+      </c>
+      <c r="H56" t="s">
+        <v>6</v>
+      </c>
+      <c r="I56" t="s">
         <v>100</v>
-      </c>
-      <c r="G56" t="s">
-        <v>6</v>
-      </c>
-      <c r="H56" t="s">
-        <v>6</v>
-      </c>
-      <c r="I56" t="s">
-        <v>101</v>
       </c>
       <c r="J56" t="s">
         <v>3</v>
@@ -2546,7 +2543,7 @@
         <v>76</v>
       </c>
       <c r="C57" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D57" t="s">
         <v>3</v>
@@ -2555,16 +2552,16 @@
         <v>6</v>
       </c>
       <c r="F57" t="s">
+        <v>99</v>
+      </c>
+      <c r="G57" t="s">
+        <v>3</v>
+      </c>
+      <c r="H57" t="s">
+        <v>3</v>
+      </c>
+      <c r="I57" t="s">
         <v>100</v>
-      </c>
-      <c r="G57" t="s">
-        <v>3</v>
-      </c>
-      <c r="H57" t="s">
-        <v>3</v>
-      </c>
-      <c r="I57" t="s">
-        <v>101</v>
       </c>
       <c r="J57" t="s">
         <v>6</v>
@@ -2578,7 +2575,7 @@
         <v>80</v>
       </c>
       <c r="C58" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D58" t="s">
         <v>2</v>
@@ -2587,7 +2584,7 @@
         <v>3</v>
       </c>
       <c r="F58" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G58" t="s">
         <v>3</v>
@@ -2596,7 +2593,7 @@
         <v>3</v>
       </c>
       <c r="I58" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J58" t="s">
         <v>2</v>
@@ -2610,7 +2607,7 @@
         <v>72</v>
       </c>
       <c r="C59" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D59" t="s">
         <v>2</v>
@@ -2619,7 +2616,7 @@
         <v>6</v>
       </c>
       <c r="F59" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G59" t="s">
         <v>3</v>
@@ -2628,7 +2625,7 @@
         <v>3</v>
       </c>
       <c r="I59" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J59" t="s">
         <v>3</v>
@@ -2642,7 +2639,7 @@
         <v>87</v>
       </c>
       <c r="C60" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D60" t="s">
         <v>2</v>
@@ -2660,7 +2657,7 @@
         <v>3</v>
       </c>
       <c r="I60" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J60" t="s">
         <v>3</v>
@@ -2674,7 +2671,7 @@
         <v>86</v>
       </c>
       <c r="C61" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D61" t="s">
         <v>2</v>
@@ -2683,7 +2680,7 @@
         <v>2</v>
       </c>
       <c r="F61" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G61" t="s">
         <v>2</v>
@@ -2692,7 +2689,7 @@
         <v>3</v>
       </c>
       <c r="I61" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J61" t="s">
         <v>2</v>
@@ -2706,7 +2703,7 @@
         <v>69</v>
       </c>
       <c r="C62" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D62" t="s">
         <v>3</v>
@@ -2715,7 +2712,7 @@
         <v>6</v>
       </c>
       <c r="F62" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G62" t="s">
         <v>6</v>
@@ -2738,7 +2735,7 @@
         <v>94</v>
       </c>
       <c r="C63" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D63" t="s">
         <v>2</v>
@@ -2747,7 +2744,7 @@
         <v>6</v>
       </c>
       <c r="F63" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G63" t="s">
         <v>6</v>
@@ -2756,7 +2753,7 @@
         <v>3</v>
       </c>
       <c r="I63" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J63" t="s">
         <v>2</v>
@@ -2770,7 +2767,7 @@
         <v>90</v>
       </c>
       <c r="C64" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D64" t="s">
         <v>2</v>
@@ -2802,7 +2799,7 @@
         <v>93</v>
       </c>
       <c r="C65" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D65" t="s">
         <v>2</v>
@@ -2820,7 +2817,7 @@
         <v>3</v>
       </c>
       <c r="I65" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J65" t="s">
         <v>2</v>
@@ -2834,7 +2831,7 @@
         <v>95</v>
       </c>
       <c r="C66" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D66" t="s">
         <v>2</v>
@@ -2843,7 +2840,7 @@
         <v>6</v>
       </c>
       <c r="F66" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G66" t="s">
         <v>3</v>
@@ -2852,7 +2849,7 @@
         <v>3</v>
       </c>
       <c r="I66" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J66" t="s">
         <v>2</v>
@@ -2866,7 +2863,7 @@
         <v>77</v>
       </c>
       <c r="C67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D67" t="s">
         <v>2</v>
@@ -2884,7 +2881,7 @@
         <v>3</v>
       </c>
       <c r="I67" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J67" t="s">
         <v>2</v>
@@ -2898,7 +2895,7 @@
         <v>92</v>
       </c>
       <c r="C68" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D68" t="s">
         <v>2</v>
@@ -2916,7 +2913,7 @@
         <v>3</v>
       </c>
       <c r="I68" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J68" t="s">
         <v>3</v>
@@ -2930,7 +2927,7 @@
         <v>71</v>
       </c>
       <c r="C69" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D69" t="s">
         <v>2</v>
@@ -2962,7 +2959,7 @@
         <v>79</v>
       </c>
       <c r="C70" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D70" t="s">
         <v>2</v>
@@ -2971,7 +2968,7 @@
         <v>3</v>
       </c>
       <c r="F70" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G70" t="s">
         <v>3</v>
@@ -2980,7 +2977,7 @@
         <v>6</v>
       </c>
       <c r="I70" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J70" t="s">
         <v>3</v>
@@ -2994,7 +2991,7 @@
         <v>38</v>
       </c>
       <c r="C71" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D71" t="s">
         <v>6</v>
@@ -3003,7 +3000,7 @@
         <v>6</v>
       </c>
       <c r="F71" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G71" t="s">
         <v>6</v>
@@ -3026,7 +3023,7 @@
         <v>43</v>
       </c>
       <c r="C72" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D72" t="s">
         <v>3</v>
@@ -3035,7 +3032,7 @@
         <v>6</v>
       </c>
       <c r="F72" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G72" t="s">
         <v>6</v>
@@ -3058,7 +3055,7 @@
         <v>46</v>
       </c>
       <c r="C73" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D73" t="s">
         <v>6</v>
@@ -3067,7 +3064,7 @@
         <v>6</v>
       </c>
       <c r="F73" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G73" t="s">
         <v>6</v>
@@ -3090,7 +3087,7 @@
         <v>55</v>
       </c>
       <c r="C74" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D74" t="s">
         <v>3</v>
@@ -3099,7 +3096,7 @@
         <v>6</v>
       </c>
       <c r="F74" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G74" t="s">
         <v>6</v>
@@ -3122,7 +3119,7 @@
         <v>56</v>
       </c>
       <c r="C75" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D75" t="s">
         <v>2</v>
@@ -3131,7 +3128,7 @@
         <v>6</v>
       </c>
       <c r="F75" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G75" t="s">
         <v>3</v>
@@ -3154,7 +3151,7 @@
         <v>35</v>
       </c>
       <c r="C76" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D76" t="s">
         <v>3</v>
@@ -3163,7 +3160,7 @@
         <v>6</v>
       </c>
       <c r="F76" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G76" t="s">
         <v>6</v>
@@ -3186,7 +3183,7 @@
         <v>52</v>
       </c>
       <c r="C77" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D77" t="s">
         <v>3</v>
@@ -3195,7 +3192,7 @@
         <v>6</v>
       </c>
       <c r="F77" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G77" t="s">
         <v>6</v>
@@ -3218,7 +3215,7 @@
         <v>54</v>
       </c>
       <c r="C78" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D78" t="s">
         <v>6</v>
@@ -3227,7 +3224,7 @@
         <v>6</v>
       </c>
       <c r="F78" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G78" t="s">
         <v>6</v>
@@ -3250,7 +3247,7 @@
         <v>39</v>
       </c>
       <c r="C79" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D79" t="s">
         <v>6</v>
@@ -3259,7 +3256,7 @@
         <v>6</v>
       </c>
       <c r="F79" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G79" t="s">
         <v>6</v>
@@ -3282,7 +3279,7 @@
         <v>51</v>
       </c>
       <c r="C80" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D80" t="s">
         <v>3</v>
@@ -3291,7 +3288,7 @@
         <v>6</v>
       </c>
       <c r="F80" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G80" t="s">
         <v>6</v>
@@ -3314,7 +3311,7 @@
         <v>40</v>
       </c>
       <c r="C81" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D81" t="s">
         <v>6</v>
@@ -3323,7 +3320,7 @@
         <v>6</v>
       </c>
       <c r="F81" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G81" t="s">
         <v>6</v>
@@ -3346,7 +3343,7 @@
         <v>41</v>
       </c>
       <c r="C82" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D82" t="s">
         <v>6</v>
@@ -3355,7 +3352,7 @@
         <v>6</v>
       </c>
       <c r="F82" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G82" t="s">
         <v>6</v>
@@ -3378,7 +3375,7 @@
         <v>44</v>
       </c>
       <c r="C83" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D83" t="s">
         <v>3</v>
@@ -3387,7 +3384,7 @@
         <v>6</v>
       </c>
       <c r="F83" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G83" t="s">
         <v>6</v>
@@ -3410,7 +3407,7 @@
         <v>37</v>
       </c>
       <c r="C84" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D84" t="s">
         <v>6</v>
@@ -3419,7 +3416,7 @@
         <v>6</v>
       </c>
       <c r="F84" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G84" t="s">
         <v>6</v>
@@ -3442,7 +3439,7 @@
         <v>42</v>
       </c>
       <c r="C85" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D85" t="s">
         <v>3</v>
@@ -3451,7 +3448,7 @@
         <v>6</v>
       </c>
       <c r="F85" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G85" t="s">
         <v>6</v>
@@ -3474,7 +3471,7 @@
         <v>34</v>
       </c>
       <c r="C86" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D86" t="s">
         <v>6</v>
@@ -3483,7 +3480,7 @@
         <v>6</v>
       </c>
       <c r="F86" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G86" t="s">
         <v>6</v>
@@ -3506,7 +3503,7 @@
         <v>58</v>
       </c>
       <c r="C87" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D87" t="s">
         <v>6</v>
@@ -3515,7 +3512,7 @@
         <v>6</v>
       </c>
       <c r="F87" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G87" t="s">
         <v>6</v>
@@ -3538,7 +3535,7 @@
         <v>48</v>
       </c>
       <c r="C88" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D88" t="s">
         <v>2</v>
@@ -3547,7 +3544,7 @@
         <v>3</v>
       </c>
       <c r="F88" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G88" t="s">
         <v>3</v>
@@ -3570,7 +3567,7 @@
         <v>53</v>
       </c>
       <c r="C89" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D89" t="s">
         <v>3</v>
@@ -3579,7 +3576,7 @@
         <v>6</v>
       </c>
       <c r="F89" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G89" t="s">
         <v>6</v>
@@ -3602,7 +3599,7 @@
         <v>57</v>
       </c>
       <c r="C90" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D90" t="s">
         <v>6</v>
@@ -3611,7 +3608,7 @@
         <v>6</v>
       </c>
       <c r="F90" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G90" t="s">
         <v>6</v>
@@ -3634,7 +3631,7 @@
         <v>36</v>
       </c>
       <c r="C91" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D91" t="s">
         <v>6</v>
@@ -3643,7 +3640,7 @@
         <v>6</v>
       </c>
       <c r="F91" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G91" t="s">
         <v>6</v>
@@ -3666,7 +3663,7 @@
         <v>50</v>
       </c>
       <c r="C92" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D92" t="s">
         <v>6</v>
@@ -3675,7 +3672,7 @@
         <v>6</v>
       </c>
       <c r="F92" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G92" t="s">
         <v>6</v>
@@ -3698,7 +3695,7 @@
         <v>45</v>
       </c>
       <c r="C93" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D93" t="s">
         <v>3</v>
@@ -3707,7 +3704,7 @@
         <v>6</v>
       </c>
       <c r="F93" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G93" t="s">
         <v>6</v>
@@ -3730,7 +3727,7 @@
         <v>49</v>
       </c>
       <c r="C94" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D94" t="s">
         <v>3</v>
@@ -3739,7 +3736,7 @@
         <v>6</v>
       </c>
       <c r="F94" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G94" t="s">
         <v>6</v>
@@ -3762,7 +3759,7 @@
         <v>47</v>
       </c>
       <c r="C95" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D95" t="s">
         <v>2</v>
@@ -3771,7 +3768,7 @@
         <v>3</v>
       </c>
       <c r="F95" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G95" t="s">
         <v>3</v>

</xml_diff>